<commit_message>
auto commit: 2026-03-21 10:11:58
</commit_message>
<xml_diff>
--- a/快乐羊毛系统/功能测试需要的文件2026.03.17/UI自动化/测试用例/登录.xlsx
+++ b/快乐羊毛系统/功能测试需要的文件2026.03.17/UI自动化/测试用例/登录.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="11925"/>
+    <workbookView windowWidth="13545" windowHeight="11925"/>
   </bookViews>
   <sheets>
     <sheet name="测试用例" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
     <t>测试步骤</t>
   </si>
   <si>
-    <t>预期结果</t>
+    <t>预期结果（断言）</t>
   </si>
   <si>
     <t>测试数据/备注</t>
@@ -845,7 +845,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -857,9 +857,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -876,9 +873,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1254,274 +1248,274 @@
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" ht="47" customHeight="1" spans="1:6">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="8" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" ht="24" spans="1:6">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="8" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" ht="48" spans="1:6">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="8" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" ht="48" spans="1:6">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="8" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6" ht="48" spans="1:6">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="8" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" ht="24" spans="1:6">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="8" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="8" ht="48" spans="1:6">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="9" ht="48" spans="1:6">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="8" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:6">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="8" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="11" ht="24" spans="1:6">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="4" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
     </row>
     <row r="13" spans="1:6">
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
     </row>
     <row r="14" spans="1:6">
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="B15" s="14"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
     </row>
     <row r="16" spans="1:6">
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
     </row>
     <row r="17" spans="2:6">
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
     </row>
     <row r="18" spans="2:6">
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
     </row>
     <row r="19" spans="2:6">
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
auto commit: 2026-03-21 14:44:44
</commit_message>
<xml_diff>
--- a/快乐羊毛系统/功能测试需要的文件2026.03.17/UI自动化/测试用例/登录.xlsx
+++ b/快乐羊毛系统/功能测试需要的文件2026.03.17/UI自动化/测试用例/登录.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13545" windowHeight="11925"/>
+    <workbookView windowWidth="27945" windowHeight="11925"/>
   </bookViews>
   <sheets>
     <sheet name="测试用例" sheetId="1" r:id="rId1"/>
@@ -1421,7 +1421,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1" spans="1:6">
+    <row r="10" ht="51" customHeight="1" spans="1:6">
       <c r="A10" s="3" t="s">
         <v>6</v>
       </c>

</xml_diff>